<commit_message>
results update after bug
</commit_message>
<xml_diff>
--- a/data/2.full_abstracting/25_12_01_full_decisions.xlsx
+++ b/data/2.full_abstracting/25_12_01_full_decisions.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unipdit-my.sharepoint.com/personal/tommaso_feraco_unipd_it/Documents/BESSI/living_SEB_review/data/2.full_abstracting/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2279" documentId="11_AD4D5CB4E552A5DACE1C647E305F51585ADEDD82" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B42F378-9D79-4B56-A548-1C414DAD819E}"/>
+  <xr:revisionPtr revIDLastSave="2281" documentId="11_AD4D5CB4E552A5DACE1C647E305F51585ADEDD82" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A4F303C-D7AD-443A-9DD0-B0530E082C02}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="-2390" yWindow="2790" windowWidth="14400" windowHeight="8170" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="basic_info" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="instructions" sheetId="3" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">basic_info!$A$1:$AE$3281</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">basic_info!$A$1:$AE$3279</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1612" uniqueCount="1515">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1571" uniqueCount="1498">
   <si>
     <t>title</t>
   </si>
@@ -4515,58 +4515,7 @@
     <t>semicolumn-separated list of topics</t>
   </si>
   <si>
-    <t>positiveschooloutcomes; academicachievement; learningfactors</t>
-  </si>
-  <si>
     <t>TF</t>
-  </si>
-  <si>
-    <t>Frontiers in Psychology</t>
-  </si>
-  <si>
-    <t>Social Psychology of Education</t>
-  </si>
-  <si>
-    <t>Sharabi, Adi and Carretti, Barbara and Cueli, Marisol Soledad and RodrÃ­guez PÃ©rez, Celestino and Pellegrino, Gerardo</t>
-  </si>
-  <si>
-    <t>Collie, Rebecca J. and Ryan, Richard M.</t>
-  </si>
-  <si>
-    <t>Autonomy support and studentsâ€™ perceived social-emotional competence: predicting parent-reported social-emotional skills</t>
-  </si>
-  <si>
-    <t>The present study tested a comprehensive model in which five social, emotional, and behavioral (SEB) skill domains (self-management, social engagement, cooperation, emotional resilience, and innovation</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.1007/s11218-025-10079-9</t>
-  </si>
-  <si>
-    <t>In this study, we investigated perceived social-emotional competence (PSEC) among 373 Australian secondary school students in relation to parent ratings of social-emotional skills, and perceived teacher and parental autonomy support. Using bifactor exploratory structural equation modelling, we examined five dimensions of PSEC (perceived competence for assertiveness, tolerance, social regulation, emotion regulation, and emotional awareness), identifying a global factor and five specific factors. Following that, we employed structural equation modelling to investigate links between these global and specific factors and five parent-reported social-emotional skills: leadership, cultural competence, teamwork, cognitive reappraisal, and capacity for emotional reflection. Global PSEC was associated positively with all skills, whereas the specific factors were, with one exception, each associated with greater parent-rated skill in a corresponding area (e.g., assertiveness with greater leadership skill; emotion awareness with reflective skills). Addressing a second aim of the research, we tested the extent to which students’ perceptions of autonomy support from teachers and parents assessed near the start of a school term were associated with both students’ PSEC and parent-rated skills assessed at the end of the term. Autonomy-supportive parenting was positively associated with global PSEC. Autonomy-supportive teaching was associated with greater levels of two specific factors: perceived competence for assertiveness and social regulation. Together, findings hold relevance to knowledge and efforts aimed at enhancing social-emotional skills among students.</t>
-  </si>
-  <si>
-    <t>Collie &amp; Ryan</t>
-  </si>
-  <si>
-    <t>Sharabi et al.</t>
-  </si>
-  <si>
-    <t>Undergraduates' achievement and satisfaction: the role of study-related factors and soft skills</t>
-  </si>
-  <si>
-    <t>https://doi.org/10.3389/fpsyg.2025.1653072</t>
-  </si>
-  <si>
-    <t>adi.sharabi@smkb.ac.il</t>
-  </si>
-  <si>
-    <t>rebecca.collie@unsw.edu.au</t>
-  </si>
-  <si>
-    <t>NO</t>
-  </si>
-  <si>
-    <t>autonomysupport</t>
   </si>
   <si>
     <t>A growing body of evidence has found that social and emotional (SE) skills are positively associated with many school-related outcomes. In recent years, the Big Five personality framework has gained support as an organizing framework for various SE skills. While many prominent taxonomies of SE skills map to the Big Five, several additional models include skills related to motivation and growth mindset that do not align with the Big Five. We examined the extent to which these constructs overlapped with SE skills organized by the Big Five framework and whether they provided incremental validity in predicting school-related outcomes. ACT test takers (N = 1755) from across the United States, mostly from high-income families and predominantly in 11th or 12th grade, completed several measures. These included a measure of SE skills as organized by the Big Five (i.e., BFI-2-S), items on school-related outcomes, measures of motivation (i.e., MSLQ, Expectancy-Value-Cost Scale, Self-Determination Scale), and a measure of growth mindset (i.e., the Growth Mindset Scale). We found that growth mindset and motivation correlated with SE skills as organized by the Big Five. These constructs also helped predict additional variance in school-related outcomes, such as GPA and ACT scores. Given the independent contributions of growth mindset and motivation, incorporating these constructs into school-based assessments, alongside SE skills, could be beneficial in supporting students. Impact Statement: The results from this study suggest that measuring growth mindset and motivation along with social and emotional skills could help to better predict which students are likely to be successful academically. From a theoretical standpoint, the current study suggests the Big Five alone may not fully capture all factors relevant for student success. Â© 2025</t>
@@ -4644,17 +4593,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
@@ -4939,7 +4885,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Foglio1"/>
-  <dimension ref="A1:AE3281"/>
+  <dimension ref="A1:AE3279"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.81640625" bestFit="1" customWidth="1"/>
@@ -5048,214 +4994,61 @@
         <v>1456</v>
       </c>
     </row>
-    <row r="2" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="6">
-        <v>45962</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D2" s="5" t="str">
-        <f t="shared" ref="D2:D59" si="0">B2&amp;""&amp;C2</f>
-        <v>0080a</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>1503</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>1502</v>
-      </c>
-      <c r="G2" s="5" t="s">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="A2" s="5">
+        <v>45992</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D2" s="4" t="str">
+        <f t="shared" ref="D2:D57" si="0">B2&amp;""&amp;C2</f>
+        <v>0088</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>1496</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1492</v>
+      </c>
+      <c r="G2" t="s">
+        <v>1491</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>1493</v>
+      </c>
+      <c r="I2" t="s">
+        <v>1494</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>1495</v>
+      </c>
+      <c r="K2" s="4">
+        <v>2025</v>
+      </c>
+      <c r="L2" t="s">
+        <v>1447</v>
+      </c>
+      <c r="O2" t="s">
+        <v>1445</v>
+      </c>
+      <c r="P2" s="6" t="s">
         <v>1497</v>
       </c>
-      <c r="H2" s="5" t="s">
-        <v>1492</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>1494</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>1501</v>
-      </c>
-      <c r="K2" s="5">
-        <v>2025</v>
-      </c>
-      <c r="L2" s="5" t="s">
-        <v>1455</v>
-      </c>
-      <c r="M2" s="5" t="s">
-        <v>1455</v>
-      </c>
-      <c r="N2" s="5" t="s">
+      <c r="AC2" t="s">
         <v>1490</v>
       </c>
-      <c r="O2" s="5" t="s">
-        <v>1486</v>
-      </c>
-      <c r="P2" s="7" t="s">
-        <v>1504</v>
-      </c>
-      <c r="Q2" s="5" t="s">
-        <v>1506</v>
-      </c>
-      <c r="R2" s="5" t="s">
-        <v>1161</v>
-      </c>
-      <c r="S2" s="5" t="s">
-        <v>1416</v>
-      </c>
-      <c r="T2" s="5">
-        <v>80</v>
-      </c>
-      <c r="U2" s="5">
-        <v>22.74</v>
-      </c>
-      <c r="V2" s="5">
-        <v>319</v>
-      </c>
-      <c r="W2" s="5" t="s">
-        <v>1166</v>
-      </c>
-      <c r="X2" s="5" t="s">
-        <v>1452</v>
-      </c>
-      <c r="Z2" s="5" t="s">
-        <v>1172</v>
-      </c>
-      <c r="AA2" s="5" t="s">
-        <v>1173</v>
-      </c>
-      <c r="AC2" s="5" t="s">
-        <v>1491</v>
-      </c>
-    </row>
-    <row r="3" spans="1:31" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="6">
-        <v>45931</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="5" t="str">
+    </row>
+    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
+      <c r="D3" t="str">
         <f t="shared" si="0"/>
-        <v>0087a</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>1498</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>1496</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>1499</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>1493</v>
-      </c>
-      <c r="I3" s="5" t="s">
-        <v>1495</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>1500</v>
-      </c>
-      <c r="K3" s="5">
-        <v>2025</v>
-      </c>
-      <c r="L3" s="5" t="s">
-        <v>1455</v>
-      </c>
-      <c r="N3" s="5" t="s">
-        <v>1507</v>
-      </c>
-      <c r="O3" s="5" t="s">
-        <v>1486</v>
-      </c>
-      <c r="P3" s="7" t="s">
-        <v>1505</v>
-      </c>
-      <c r="Q3" s="5" t="s">
-        <v>1506</v>
-      </c>
-      <c r="R3" s="5" t="s">
-        <v>1161</v>
-      </c>
-      <c r="S3" s="5" t="s">
-        <v>1188</v>
-      </c>
-      <c r="T3" s="5">
-        <v>51</v>
-      </c>
-      <c r="U3" s="5">
-        <v>14</v>
-      </c>
-      <c r="V3" s="5">
-        <v>373</v>
-      </c>
-      <c r="W3" s="5" t="s">
-        <v>1165</v>
-      </c>
-      <c r="X3" s="5" t="s">
-        <v>1452</v>
-      </c>
-      <c r="Z3" s="5" t="s">
-        <v>1459</v>
-      </c>
-      <c r="AA3" s="5" t="s">
-        <v>1173</v>
-      </c>
-      <c r="AC3" s="5" t="s">
-        <v>1491</v>
+        <v/>
       </c>
     </row>
     <row r="4" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A4" s="8">
-        <v>45992</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="D4" s="5" t="str">
+      <c r="D4" t="str">
         <f t="shared" si="0"/>
-        <v>0088</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>1513</v>
-      </c>
-      <c r="F4" t="s">
-        <v>1509</v>
-      </c>
-      <c r="G4" t="s">
-        <v>1508</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>1510</v>
-      </c>
-      <c r="I4" t="s">
-        <v>1511</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>1512</v>
-      </c>
-      <c r="K4" s="5">
-        <v>2025</v>
-      </c>
-      <c r="L4" t="s">
-        <v>1447</v>
-      </c>
-      <c r="O4" t="s">
-        <v>1445</v>
-      </c>
-      <c r="P4" s="9" t="s">
-        <v>1514</v>
-      </c>
-      <c r="AC4" t="s">
-        <v>1491</v>
+        <v/>
       </c>
     </row>
     <row r="5" spans="1:31" x14ac:dyDescent="0.35">
@@ -5578,19 +5371,19 @@
     </row>
     <row r="58" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D58" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="D58:D121" si="1">B58&amp;""&amp;C58</f>
         <v/>
       </c>
     </row>
     <row r="59" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D59" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="60" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D60" t="str">
-        <f t="shared" ref="D60:D123" si="1">B60&amp;""&amp;C60</f>
+        <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
@@ -5962,19 +5755,19 @@
     </row>
     <row r="122" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D122" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="D122:D185" si="2">B122&amp;""&amp;C122</f>
         <v/>
       </c>
     </row>
     <row r="123" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D123" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="124" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D124" t="str">
-        <f t="shared" ref="D124:D187" si="2">B124&amp;""&amp;C124</f>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -6346,19 +6139,19 @@
     </row>
     <row r="186" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D186" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="D186:D249" si="3">B186&amp;""&amp;C186</f>
         <v/>
       </c>
     </row>
     <row r="187" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D187" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
     <row r="188" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D188" t="str">
-        <f t="shared" ref="D188:D251" si="3">B188&amp;""&amp;C188</f>
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -6730,19 +6523,19 @@
     </row>
     <row r="250" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D250" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="D250:D313" si="4">B250&amp;""&amp;C250</f>
         <v/>
       </c>
     </row>
     <row r="251" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D251" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
     <row r="252" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D252" t="str">
-        <f t="shared" ref="D252:D315" si="4">B252&amp;""&amp;C252</f>
+        <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
@@ -7114,19 +6907,19 @@
     </row>
     <row r="314" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D314" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" ref="D314:D377" si="5">B314&amp;""&amp;C314</f>
         <v/>
       </c>
     </row>
     <row r="315" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D315" t="str">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
     <row r="316" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D316" t="str">
-        <f t="shared" ref="D316:D379" si="5">B316&amp;""&amp;C316</f>
+        <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
@@ -7498,19 +7291,19 @@
     </row>
     <row r="378" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D378" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" ref="D378:D441" si="6">B378&amp;""&amp;C378</f>
         <v/>
       </c>
     </row>
     <row r="379" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D379" t="str">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
     <row r="380" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D380" t="str">
-        <f t="shared" ref="D380:D443" si="6">B380&amp;""&amp;C380</f>
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
@@ -7882,19 +7675,19 @@
     </row>
     <row r="442" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D442" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" ref="D442:D505" si="7">B442&amp;""&amp;C442</f>
         <v/>
       </c>
     </row>
     <row r="443" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D443" t="str">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
     <row r="444" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D444" t="str">
-        <f t="shared" ref="D444:D507" si="7">B444&amp;""&amp;C444</f>
+        <f t="shared" si="7"/>
         <v/>
       </c>
     </row>
@@ -8266,19 +8059,19 @@
     </row>
     <row r="506" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D506" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="D506:D569" si="8">B506&amp;""&amp;C506</f>
         <v/>
       </c>
     </row>
     <row r="507" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D507" t="str">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
     <row r="508" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D508" t="str">
-        <f t="shared" ref="D508:D571" si="8">B508&amp;""&amp;C508</f>
+        <f t="shared" si="8"/>
         <v/>
       </c>
     </row>
@@ -8650,19 +8443,19 @@
     </row>
     <row r="570" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D570" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" ref="D570:D633" si="9">B570&amp;""&amp;C570</f>
         <v/>
       </c>
     </row>
     <row r="571" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D571" t="str">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v/>
       </c>
     </row>
     <row r="572" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D572" t="str">
-        <f t="shared" ref="D572:D635" si="9">B572&amp;""&amp;C572</f>
+        <f t="shared" si="9"/>
         <v/>
       </c>
     </row>
@@ -9034,19 +8827,19 @@
     </row>
     <row r="634" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D634" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" ref="D634:D697" si="10">B634&amp;""&amp;C634</f>
         <v/>
       </c>
     </row>
     <row r="635" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D635" t="str">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
     <row r="636" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D636" t="str">
-        <f t="shared" ref="D636:D699" si="10">B636&amp;""&amp;C636</f>
+        <f t="shared" si="10"/>
         <v/>
       </c>
     </row>
@@ -9418,19 +9211,19 @@
     </row>
     <row r="698" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D698" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" ref="D698:D761" si="11">B698&amp;""&amp;C698</f>
         <v/>
       </c>
     </row>
     <row r="699" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D699" t="str">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
     <row r="700" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D700" t="str">
-        <f t="shared" ref="D700:D763" si="11">B700&amp;""&amp;C700</f>
+        <f t="shared" si="11"/>
         <v/>
       </c>
     </row>
@@ -9802,19 +9595,19 @@
     </row>
     <row r="762" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D762" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" ref="D762:D825" si="12">B762&amp;""&amp;C762</f>
         <v/>
       </c>
     </row>
     <row r="763" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D763" t="str">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v/>
       </c>
     </row>
     <row r="764" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D764" t="str">
-        <f t="shared" ref="D764:D827" si="12">B764&amp;""&amp;C764</f>
+        <f t="shared" si="12"/>
         <v/>
       </c>
     </row>
@@ -10186,19 +9979,19 @@
     </row>
     <row r="826" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D826" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" ref="D826:D889" si="13">B826&amp;""&amp;C826</f>
         <v/>
       </c>
     </row>
     <row r="827" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D827" t="str">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v/>
       </c>
     </row>
     <row r="828" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D828" t="str">
-        <f t="shared" ref="D828:D891" si="13">B828&amp;""&amp;C828</f>
+        <f t="shared" si="13"/>
         <v/>
       </c>
     </row>
@@ -10570,19 +10363,19 @@
     </row>
     <row r="890" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D890" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" ref="D890:D953" si="14">B890&amp;""&amp;C890</f>
         <v/>
       </c>
     </row>
     <row r="891" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D891" t="str">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
     <row r="892" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D892" t="str">
-        <f t="shared" ref="D892:D955" si="14">B892&amp;""&amp;C892</f>
+        <f t="shared" si="14"/>
         <v/>
       </c>
     </row>
@@ -10954,19 +10747,19 @@
     </row>
     <row r="954" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D954" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" ref="D954:D1017" si="15">B954&amp;""&amp;C954</f>
         <v/>
       </c>
     </row>
     <row r="955" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D955" t="str">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v/>
       </c>
     </row>
     <row r="956" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D956" t="str">
-        <f t="shared" ref="D956:D1019" si="15">B956&amp;""&amp;C956</f>
+        <f t="shared" si="15"/>
         <v/>
       </c>
     </row>
@@ -11338,19 +11131,19 @@
     </row>
     <row r="1018" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1018" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" ref="D1018:D1081" si="16">B1018&amp;""&amp;C1018</f>
         <v/>
       </c>
     </row>
     <row r="1019" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1019" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="16"/>
         <v/>
       </c>
     </row>
     <row r="1020" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1020" t="str">
-        <f t="shared" ref="D1020:D1083" si="16">B1020&amp;""&amp;C1020</f>
+        <f t="shared" si="16"/>
         <v/>
       </c>
     </row>
@@ -11722,19 +11515,19 @@
     </row>
     <row r="1082" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1082" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" ref="D1082:D1145" si="17">B1082&amp;""&amp;C1082</f>
         <v/>
       </c>
     </row>
     <row r="1083" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1083" t="str">
-        <f t="shared" si="16"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
     </row>
     <row r="1084" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1084" t="str">
-        <f t="shared" ref="D1084:D1147" si="17">B1084&amp;""&amp;C1084</f>
+        <f t="shared" si="17"/>
         <v/>
       </c>
     </row>
@@ -12106,19 +11899,19 @@
     </row>
     <row r="1146" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1146" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" ref="D1146:D1209" si="18">B1146&amp;""&amp;C1146</f>
         <v/>
       </c>
     </row>
     <row r="1147" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1147" t="str">
-        <f t="shared" si="17"/>
+        <f t="shared" si="18"/>
         <v/>
       </c>
     </row>
     <row r="1148" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1148" t="str">
-        <f t="shared" ref="D1148:D1211" si="18">B1148&amp;""&amp;C1148</f>
+        <f t="shared" si="18"/>
         <v/>
       </c>
     </row>
@@ -12490,19 +12283,19 @@
     </row>
     <row r="1210" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1210" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" ref="D1210:D1273" si="19">B1210&amp;""&amp;C1210</f>
         <v/>
       </c>
     </row>
     <row r="1211" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1211" t="str">
-        <f t="shared" si="18"/>
+        <f t="shared" si="19"/>
         <v/>
       </c>
     </row>
     <row r="1212" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1212" t="str">
-        <f t="shared" ref="D1212:D1275" si="19">B1212&amp;""&amp;C1212</f>
+        <f t="shared" si="19"/>
         <v/>
       </c>
     </row>
@@ -12874,19 +12667,19 @@
     </row>
     <row r="1274" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1274" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" ref="D1274:D1337" si="20">B1274&amp;""&amp;C1274</f>
         <v/>
       </c>
     </row>
     <row r="1275" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1275" t="str">
-        <f t="shared" si="19"/>
+        <f t="shared" si="20"/>
         <v/>
       </c>
     </row>
     <row r="1276" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1276" t="str">
-        <f t="shared" ref="D1276:D1339" si="20">B1276&amp;""&amp;C1276</f>
+        <f t="shared" si="20"/>
         <v/>
       </c>
     </row>
@@ -13258,19 +13051,19 @@
     </row>
     <row r="1338" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1338" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" ref="D1338:D1401" si="21">B1338&amp;""&amp;C1338</f>
         <v/>
       </c>
     </row>
     <row r="1339" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1339" t="str">
-        <f t="shared" si="20"/>
+        <f t="shared" si="21"/>
         <v/>
       </c>
     </row>
     <row r="1340" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1340" t="str">
-        <f t="shared" ref="D1340:D1403" si="21">B1340&amp;""&amp;C1340</f>
+        <f t="shared" si="21"/>
         <v/>
       </c>
     </row>
@@ -13642,19 +13435,19 @@
     </row>
     <row r="1402" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1402" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" ref="D1402:D1465" si="22">B1402&amp;""&amp;C1402</f>
         <v/>
       </c>
     </row>
     <row r="1403" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1403" t="str">
-        <f t="shared" si="21"/>
+        <f t="shared" si="22"/>
         <v/>
       </c>
     </row>
     <row r="1404" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1404" t="str">
-        <f t="shared" ref="D1404:D1467" si="22">B1404&amp;""&amp;C1404</f>
+        <f t="shared" si="22"/>
         <v/>
       </c>
     </row>
@@ -14026,19 +13819,19 @@
     </row>
     <row r="1466" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1466" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" ref="D1466:D1529" si="23">B1466&amp;""&amp;C1466</f>
         <v/>
       </c>
     </row>
     <row r="1467" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1467" t="str">
-        <f t="shared" si="22"/>
+        <f t="shared" si="23"/>
         <v/>
       </c>
     </row>
     <row r="1468" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1468" t="str">
-        <f t="shared" ref="D1468:D1531" si="23">B1468&amp;""&amp;C1468</f>
+        <f t="shared" si="23"/>
         <v/>
       </c>
     </row>
@@ -14410,19 +14203,19 @@
     </row>
     <row r="1530" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1530" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" ref="D1530:D1593" si="24">B1530&amp;""&amp;C1530</f>
         <v/>
       </c>
     </row>
     <row r="1531" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1531" t="str">
-        <f t="shared" si="23"/>
+        <f t="shared" si="24"/>
         <v/>
       </c>
     </row>
     <row r="1532" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1532" t="str">
-        <f t="shared" ref="D1532:D1595" si="24">B1532&amp;""&amp;C1532</f>
+        <f t="shared" si="24"/>
         <v/>
       </c>
     </row>
@@ -14794,19 +14587,19 @@
     </row>
     <row r="1594" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1594" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" ref="D1594:D1657" si="25">B1594&amp;""&amp;C1594</f>
         <v/>
       </c>
     </row>
     <row r="1595" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1595" t="str">
-        <f t="shared" si="24"/>
+        <f t="shared" si="25"/>
         <v/>
       </c>
     </row>
     <row r="1596" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1596" t="str">
-        <f t="shared" ref="D1596:D1659" si="25">B1596&amp;""&amp;C1596</f>
+        <f t="shared" si="25"/>
         <v/>
       </c>
     </row>
@@ -15178,19 +14971,19 @@
     </row>
     <row r="1658" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1658" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" ref="D1658:D1721" si="26">B1658&amp;""&amp;C1658</f>
         <v/>
       </c>
     </row>
     <row r="1659" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1659" t="str">
-        <f t="shared" si="25"/>
+        <f t="shared" si="26"/>
         <v/>
       </c>
     </row>
     <row r="1660" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1660" t="str">
-        <f t="shared" ref="D1660:D1723" si="26">B1660&amp;""&amp;C1660</f>
+        <f t="shared" si="26"/>
         <v/>
       </c>
     </row>
@@ -15562,19 +15355,19 @@
     </row>
     <row r="1722" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1722" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" ref="D1722:D1785" si="27">B1722&amp;""&amp;C1722</f>
         <v/>
       </c>
     </row>
     <row r="1723" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1723" t="str">
-        <f t="shared" si="26"/>
+        <f t="shared" si="27"/>
         <v/>
       </c>
     </row>
     <row r="1724" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1724" t="str">
-        <f t="shared" ref="D1724:D1787" si="27">B1724&amp;""&amp;C1724</f>
+        <f t="shared" si="27"/>
         <v/>
       </c>
     </row>
@@ -15946,19 +15739,19 @@
     </row>
     <row r="1786" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1786" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" ref="D1786:D1849" si="28">B1786&amp;""&amp;C1786</f>
         <v/>
       </c>
     </row>
     <row r="1787" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1787" t="str">
-        <f t="shared" si="27"/>
+        <f t="shared" si="28"/>
         <v/>
       </c>
     </row>
     <row r="1788" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1788" t="str">
-        <f t="shared" ref="D1788:D1851" si="28">B1788&amp;""&amp;C1788</f>
+        <f t="shared" si="28"/>
         <v/>
       </c>
     </row>
@@ -16330,19 +16123,19 @@
     </row>
     <row r="1850" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1850" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" ref="D1850:D1913" si="29">B1850&amp;""&amp;C1850</f>
         <v/>
       </c>
     </row>
     <row r="1851" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1851" t="str">
-        <f t="shared" si="28"/>
+        <f t="shared" si="29"/>
         <v/>
       </c>
     </row>
     <row r="1852" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1852" t="str">
-        <f t="shared" ref="D1852:D1915" si="29">B1852&amp;""&amp;C1852</f>
+        <f t="shared" si="29"/>
         <v/>
       </c>
     </row>
@@ -16714,19 +16507,19 @@
     </row>
     <row r="1914" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1914" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" ref="D1914:D1977" si="30">B1914&amp;""&amp;C1914</f>
         <v/>
       </c>
     </row>
     <row r="1915" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1915" t="str">
-        <f t="shared" si="29"/>
+        <f t="shared" si="30"/>
         <v/>
       </c>
     </row>
     <row r="1916" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1916" t="str">
-        <f t="shared" ref="D1916:D1979" si="30">B1916&amp;""&amp;C1916</f>
+        <f t="shared" si="30"/>
         <v/>
       </c>
     </row>
@@ -17098,19 +16891,19 @@
     </row>
     <row r="1978" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1978" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" ref="D1978:D2041" si="31">B1978&amp;""&amp;C1978</f>
         <v/>
       </c>
     </row>
     <row r="1979" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1979" t="str">
-        <f t="shared" si="30"/>
+        <f t="shared" si="31"/>
         <v/>
       </c>
     </row>
     <row r="1980" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D1980" t="str">
-        <f t="shared" ref="D1980:D2043" si="31">B1980&amp;""&amp;C1980</f>
+        <f t="shared" si="31"/>
         <v/>
       </c>
     </row>
@@ -17482,19 +17275,19 @@
     </row>
     <row r="2042" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2042" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" ref="D2042:D2105" si="32">B2042&amp;""&amp;C2042</f>
         <v/>
       </c>
     </row>
     <row r="2043" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2043" t="str">
-        <f t="shared" si="31"/>
+        <f t="shared" si="32"/>
         <v/>
       </c>
     </row>
     <row r="2044" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2044" t="str">
-        <f t="shared" ref="D2044:D2107" si="32">B2044&amp;""&amp;C2044</f>
+        <f t="shared" si="32"/>
         <v/>
       </c>
     </row>
@@ -17866,19 +17659,19 @@
     </row>
     <row r="2106" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2106" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" ref="D2106:D2169" si="33">B2106&amp;""&amp;C2106</f>
         <v/>
       </c>
     </row>
     <row r="2107" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2107" t="str">
-        <f t="shared" si="32"/>
+        <f t="shared" si="33"/>
         <v/>
       </c>
     </row>
     <row r="2108" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2108" t="str">
-        <f t="shared" ref="D2108:D2171" si="33">B2108&amp;""&amp;C2108</f>
+        <f t="shared" si="33"/>
         <v/>
       </c>
     </row>
@@ -18250,19 +18043,19 @@
     </row>
     <row r="2170" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2170" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" ref="D2170:D2233" si="34">B2170&amp;""&amp;C2170</f>
         <v/>
       </c>
     </row>
     <row r="2171" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2171" t="str">
-        <f t="shared" si="33"/>
+        <f t="shared" si="34"/>
         <v/>
       </c>
     </row>
     <row r="2172" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2172" t="str">
-        <f t="shared" ref="D2172:D2235" si="34">B2172&amp;""&amp;C2172</f>
+        <f t="shared" si="34"/>
         <v/>
       </c>
     </row>
@@ -18634,19 +18427,19 @@
     </row>
     <row r="2234" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2234" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" ref="D2234:D2297" si="35">B2234&amp;""&amp;C2234</f>
         <v/>
       </c>
     </row>
     <row r="2235" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2235" t="str">
-        <f t="shared" si="34"/>
+        <f t="shared" si="35"/>
         <v/>
       </c>
     </row>
     <row r="2236" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2236" t="str">
-        <f t="shared" ref="D2236:D2299" si="35">B2236&amp;""&amp;C2236</f>
+        <f t="shared" si="35"/>
         <v/>
       </c>
     </row>
@@ -19018,19 +18811,19 @@
     </row>
     <row r="2298" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2298" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" ref="D2298:D2361" si="36">B2298&amp;""&amp;C2298</f>
         <v/>
       </c>
     </row>
     <row r="2299" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2299" t="str">
-        <f t="shared" si="35"/>
+        <f t="shared" si="36"/>
         <v/>
       </c>
     </row>
     <row r="2300" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2300" t="str">
-        <f t="shared" ref="D2300:D2363" si="36">B2300&amp;""&amp;C2300</f>
+        <f t="shared" si="36"/>
         <v/>
       </c>
     </row>
@@ -19402,19 +19195,19 @@
     </row>
     <row r="2362" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2362" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" ref="D2362:D2425" si="37">B2362&amp;""&amp;C2362</f>
         <v/>
       </c>
     </row>
     <row r="2363" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2363" t="str">
-        <f t="shared" si="36"/>
+        <f t="shared" si="37"/>
         <v/>
       </c>
     </row>
     <row r="2364" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2364" t="str">
-        <f t="shared" ref="D2364:D2427" si="37">B2364&amp;""&amp;C2364</f>
+        <f t="shared" si="37"/>
         <v/>
       </c>
     </row>
@@ -19786,19 +19579,19 @@
     </row>
     <row r="2426" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2426" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" ref="D2426:D2489" si="38">B2426&amp;""&amp;C2426</f>
         <v/>
       </c>
     </row>
     <row r="2427" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2427" t="str">
-        <f t="shared" si="37"/>
+        <f t="shared" si="38"/>
         <v/>
       </c>
     </row>
     <row r="2428" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2428" t="str">
-        <f t="shared" ref="D2428:D2491" si="38">B2428&amp;""&amp;C2428</f>
+        <f t="shared" si="38"/>
         <v/>
       </c>
     </row>
@@ -20170,19 +19963,19 @@
     </row>
     <row r="2490" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2490" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" ref="D2490:D2553" si="39">B2490&amp;""&amp;C2490</f>
         <v/>
       </c>
     </row>
     <row r="2491" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2491" t="str">
-        <f t="shared" si="38"/>
+        <f t="shared" si="39"/>
         <v/>
       </c>
     </row>
     <row r="2492" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2492" t="str">
-        <f t="shared" ref="D2492:D2555" si="39">B2492&amp;""&amp;C2492</f>
+        <f t="shared" si="39"/>
         <v/>
       </c>
     </row>
@@ -20554,19 +20347,19 @@
     </row>
     <row r="2554" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2554" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" ref="D2554:D2617" si="40">B2554&amp;""&amp;C2554</f>
         <v/>
       </c>
     </row>
     <row r="2555" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2555" t="str">
-        <f t="shared" si="39"/>
+        <f t="shared" si="40"/>
         <v/>
       </c>
     </row>
     <row r="2556" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2556" t="str">
-        <f t="shared" ref="D2556:D2619" si="40">B2556&amp;""&amp;C2556</f>
+        <f t="shared" si="40"/>
         <v/>
       </c>
     </row>
@@ -20938,19 +20731,19 @@
     </row>
     <row r="2618" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2618" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" ref="D2618:D2681" si="41">B2618&amp;""&amp;C2618</f>
         <v/>
       </c>
     </row>
     <row r="2619" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2619" t="str">
-        <f t="shared" si="40"/>
+        <f t="shared" si="41"/>
         <v/>
       </c>
     </row>
     <row r="2620" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2620" t="str">
-        <f t="shared" ref="D2620:D2683" si="41">B2620&amp;""&amp;C2620</f>
+        <f t="shared" si="41"/>
         <v/>
       </c>
     </row>
@@ -21322,19 +21115,19 @@
     </row>
     <row r="2682" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2682" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" ref="D2682:D2745" si="42">B2682&amp;""&amp;C2682</f>
         <v/>
       </c>
     </row>
     <row r="2683" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2683" t="str">
-        <f t="shared" si="41"/>
+        <f t="shared" si="42"/>
         <v/>
       </c>
     </row>
     <row r="2684" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2684" t="str">
-        <f t="shared" ref="D2684:D2747" si="42">B2684&amp;""&amp;C2684</f>
+        <f t="shared" si="42"/>
         <v/>
       </c>
     </row>
@@ -21706,19 +21499,19 @@
     </row>
     <row r="2746" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2746" t="str">
-        <f t="shared" si="42"/>
+        <f t="shared" ref="D2746:D2809" si="43">B2746&amp;""&amp;C2746</f>
         <v/>
       </c>
     </row>
     <row r="2747" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2747" t="str">
-        <f t="shared" si="42"/>
+        <f t="shared" si="43"/>
         <v/>
       </c>
     </row>
     <row r="2748" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2748" t="str">
-        <f t="shared" ref="D2748:D2811" si="43">B2748&amp;""&amp;C2748</f>
+        <f t="shared" si="43"/>
         <v/>
       </c>
     </row>
@@ -22090,19 +21883,19 @@
     </row>
     <row r="2810" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2810" t="str">
-        <f t="shared" si="43"/>
+        <f t="shared" ref="D2810:D2873" si="44">B2810&amp;""&amp;C2810</f>
         <v/>
       </c>
     </row>
     <row r="2811" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2811" t="str">
-        <f t="shared" si="43"/>
+        <f t="shared" si="44"/>
         <v/>
       </c>
     </row>
     <row r="2812" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2812" t="str">
-        <f t="shared" ref="D2812:D2875" si="44">B2812&amp;""&amp;C2812</f>
+        <f t="shared" si="44"/>
         <v/>
       </c>
     </row>
@@ -22474,19 +22267,19 @@
     </row>
     <row r="2874" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2874" t="str">
-        <f t="shared" si="44"/>
+        <f t="shared" ref="D2874:D2937" si="45">B2874&amp;""&amp;C2874</f>
         <v/>
       </c>
     </row>
     <row r="2875" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2875" t="str">
-        <f t="shared" si="44"/>
+        <f t="shared" si="45"/>
         <v/>
       </c>
     </row>
     <row r="2876" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2876" t="str">
-        <f t="shared" ref="D2876:D2939" si="45">B2876&amp;""&amp;C2876</f>
+        <f t="shared" si="45"/>
         <v/>
       </c>
     </row>
@@ -22858,19 +22651,19 @@
     </row>
     <row r="2938" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2938" t="str">
-        <f t="shared" si="45"/>
+        <f t="shared" ref="D2938:D3001" si="46">B2938&amp;""&amp;C2938</f>
         <v/>
       </c>
     </row>
     <row r="2939" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2939" t="str">
-        <f t="shared" si="45"/>
+        <f t="shared" si="46"/>
         <v/>
       </c>
     </row>
     <row r="2940" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D2940" t="str">
-        <f t="shared" ref="D2940:D3003" si="46">B2940&amp;""&amp;C2940</f>
+        <f t="shared" si="46"/>
         <v/>
       </c>
     </row>
@@ -23242,19 +23035,19 @@
     </row>
     <row r="3002" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D3002" t="str">
-        <f t="shared" si="46"/>
+        <f t="shared" ref="D3002:D3065" si="47">B3002&amp;""&amp;C3002</f>
         <v/>
       </c>
     </row>
     <row r="3003" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D3003" t="str">
-        <f t="shared" si="46"/>
+        <f t="shared" si="47"/>
         <v/>
       </c>
     </row>
     <row r="3004" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D3004" t="str">
-        <f t="shared" ref="D3004:D3067" si="47">B3004&amp;""&amp;C3004</f>
+        <f t="shared" si="47"/>
         <v/>
       </c>
     </row>
@@ -23626,19 +23419,19 @@
     </row>
     <row r="3066" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D3066" t="str">
-        <f t="shared" si="47"/>
+        <f t="shared" ref="D3066:D3129" si="48">B3066&amp;""&amp;C3066</f>
         <v/>
       </c>
     </row>
     <row r="3067" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D3067" t="str">
-        <f t="shared" si="47"/>
+        <f t="shared" si="48"/>
         <v/>
       </c>
     </row>
     <row r="3068" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D3068" t="str">
-        <f t="shared" ref="D3068:D3131" si="48">B3068&amp;""&amp;C3068</f>
+        <f t="shared" si="48"/>
         <v/>
       </c>
     </row>
@@ -24010,19 +23803,19 @@
     </row>
     <row r="3130" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D3130" t="str">
-        <f t="shared" si="48"/>
+        <f t="shared" ref="D3130:D3193" si="49">B3130&amp;""&amp;C3130</f>
         <v/>
       </c>
     </row>
     <row r="3131" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D3131" t="str">
-        <f t="shared" si="48"/>
+        <f t="shared" si="49"/>
         <v/>
       </c>
     </row>
     <row r="3132" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D3132" t="str">
-        <f t="shared" ref="D3132:D3195" si="49">B3132&amp;""&amp;C3132</f>
+        <f t="shared" si="49"/>
         <v/>
       </c>
     </row>
@@ -24394,19 +24187,19 @@
     </row>
     <row r="3194" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D3194" t="str">
-        <f t="shared" si="49"/>
+        <f t="shared" ref="D3194:D3257" si="50">B3194&amp;""&amp;C3194</f>
         <v/>
       </c>
     </row>
     <row r="3195" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D3195" t="str">
-        <f t="shared" si="49"/>
+        <f t="shared" si="50"/>
         <v/>
       </c>
     </row>
     <row r="3196" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D3196" t="str">
-        <f t="shared" ref="D3196:D3259" si="50">B3196&amp;""&amp;C3196</f>
+        <f t="shared" si="50"/>
         <v/>
       </c>
     </row>
@@ -24778,19 +24571,19 @@
     </row>
     <row r="3258" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D3258" t="str">
-        <f t="shared" si="50"/>
+        <f t="shared" ref="D3258:D3279" si="51">B3258&amp;""&amp;C3258</f>
         <v/>
       </c>
     </row>
     <row r="3259" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D3259" t="str">
-        <f t="shared" si="50"/>
+        <f t="shared" si="51"/>
         <v/>
       </c>
     </row>
     <row r="3260" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D3260" t="str">
-        <f t="shared" ref="D3260:D3281" si="51">B3260&amp;""&amp;C3260</f>
+        <f t="shared" si="51"/>
         <v/>
       </c>
     </row>
@@ -24908,37 +24701,21 @@
         <v/>
       </c>
     </row>
-    <row r="3280" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D3280" t="str">
-        <f t="shared" si="51"/>
-        <v/>
-      </c>
-    </row>
-    <row r="3281" spans="4:4" x14ac:dyDescent="0.35">
-      <c r="D3281" t="str">
-        <f t="shared" si="51"/>
-        <v/>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:AE3281" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:AE3279" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K1297" xr:uid="{F8524D51-D2D8-47F0-889D-CF24F2B60A7D}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2:K1295" xr:uid="{F8524D51-D2D8-47F0-889D-CF24F2B60A7D}">
       <formula1>2020</formula1>
       <formula2>2040</formula2>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="E3" r:id="rId1" xr:uid="{47C16BF6-EC26-4776-A475-629192EF7EFD}"/>
-    <hyperlink ref="E2" r:id="rId2" xr:uid="{E7A087AC-B4C3-4F56-9A4F-58CF0DD6ED79}"/>
-    <hyperlink ref="P2" r:id="rId3" xr:uid="{8ED2E0F0-DA5F-4D40-A272-EC073B27433B}"/>
-    <hyperlink ref="P3" r:id="rId4" xr:uid="{FB02A930-21F9-4B83-ACDA-8640ED559FEE}"/>
-    <hyperlink ref="E4" r:id="rId5" xr:uid="{1D0679E6-8485-4C3F-8464-66578ED8C489}"/>
-    <hyperlink ref="P4" r:id="rId6" xr:uid="{6C8B467C-7DB6-45A1-8488-901665DE330A}"/>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{1D0679E6-8485-4C3F-8464-66578ED8C489}"/>
+    <hyperlink ref="P2" r:id="rId2" xr:uid="{6C8B467C-7DB6-45A1-8488-901665DE330A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="13">
@@ -24946,79 +24723,79 @@
           <x14:formula1>
             <xm:f>options!$K$2:$K$35</xm:f>
           </x14:formula1>
-          <xm:sqref>N4:N2835</xm:sqref>
+          <xm:sqref>N2:N2833</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{BE656A4B-9C86-4B7C-8372-C393037AC66D}">
           <x14:formula1>
             <xm:f>options!$T$2:$T$18</xm:f>
           </x14:formula1>
-          <xm:sqref>W2:W2588</xm:sqref>
+          <xm:sqref>W2:W2586</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{BEBF39FF-702B-4ABB-A589-6D4D7378CF4B}">
           <x14:formula1>
             <xm:f>options!$A$2:$A$112121</xm:f>
           </x14:formula1>
-          <xm:sqref>B2:B3279</xm:sqref>
+          <xm:sqref>B2:B3277</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{457573A4-3B1E-4F5B-99D6-3289E91A02EE}">
           <x14:formula1>
             <xm:f>options!$L$2:$L$7</xm:f>
           </x14:formula1>
-          <xm:sqref>O2:O2563</xm:sqref>
+          <xm:sqref>O2:O2561</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{ABFFB021-3A02-409D-9301-E0134C4E0168}">
           <x14:formula1>
             <xm:f>options!$I$2:$I$19</xm:f>
           </x14:formula1>
-          <xm:sqref>L2:L2893</xm:sqref>
+          <xm:sqref>L2:L2891</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{73622D16-B875-48DA-8FEF-B515FBFE0CD9}">
           <x14:formula1>
             <xm:f>options!$B$2:$B$22</xm:f>
           </x14:formula1>
-          <xm:sqref>C2:C2803</xm:sqref>
+          <xm:sqref>C2:C2801</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{EFCAB99E-06E1-41AD-A61B-D5D0CA9D5E9E}">
           <x14:formula1>
             <xm:f>options!$O$2:$O$16</xm:f>
           </x14:formula1>
-          <xm:sqref>R2:R3044</xm:sqref>
+          <xm:sqref>R2:R3042</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{1ECEBC84-E5EE-4D00-8FBF-A12F4235A6AE}">
           <x14:formula1>
             <xm:f>options!$P$2:$P$465</xm:f>
           </x14:formula1>
-          <xm:sqref>S2:S3513</xm:sqref>
+          <xm:sqref>S2:S3511</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A4CB52C2-24DD-480D-9C81-281827D0352F}">
           <x14:formula1>
             <xm:f>options!$W$2:$W$37</xm:f>
           </x14:formula1>
-          <xm:sqref>Z2:Z2738</xm:sqref>
+          <xm:sqref>Z2:Z2736</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{343D6D5F-6D69-4FB4-BDFA-B2BDA31BAC91}">
           <x14:formula1>
             <xm:f>options!$X$2:$X$24</xm:f>
           </x14:formula1>
-          <xm:sqref>AA2:AA2913</xm:sqref>
+          <xm:sqref>AA2:AA2911</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{ABF61035-FDD9-4029-BEFD-117D3A689719}">
           <x14:formula1>
             <xm:f>options!$Y$2:$Y$16</xm:f>
           </x14:formula1>
-          <xm:sqref>AB2:AB3515</xm:sqref>
+          <xm:sqref>AB2:AB3513</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5EDCACA3-D906-4B8C-A7FB-4512358B78BB}">
           <x14:formula1>
             <xm:f>options!$U$2:$U$8</xm:f>
           </x14:formula1>
-          <xm:sqref>X2:X3318</xm:sqref>
+          <xm:sqref>X2:X3316</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{83972B6B-CA01-43FD-BEFD-AAE363E3BAA0}">
           <x14:formula1>
             <xm:f>options!$J$2:$J$27</xm:f>
           </x14:formula1>
-          <xm:sqref>M2:M3505</xm:sqref>
+          <xm:sqref>M2:M3503</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>